<commit_message>
LCO Anpassungen in ersten Methanol Modellen
</commit_message>
<xml_diff>
--- a/Methanol/Methanol_Bio_H2_Brownfield_Höchst/Datenbank.xlsx
+++ b/Methanol/Methanol_Bio_H2_Brownfield_Höchst/Datenbank.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Arbeit\06-FENES\09-P2X3\FENES_P2X\Methanol\Methanol_Bio_H2_Brownfield_Höchst\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DA67718-C718-4F17-88A2-C39981AF1814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11A6760B-2B74-408C-9E44-9129830ECE21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-53868" yWindow="3444" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datenauswahl" sheetId="1" r:id="rId1"/>
@@ -180,7 +180,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="392">
   <si>
     <t>PEM Elektrolyse</t>
   </si>
@@ -865,12 +865,6 @@
     <t>calc_cost_h2</t>
   </si>
   <si>
-    <t>calc_einnahmen_stromverkauf_schattenvariable</t>
-  </si>
-  <si>
-    <t>Schattenvariable Einnahmen Stromverkauf</t>
-  </si>
-  <si>
     <t>Methanolsynthese</t>
   </si>
   <si>
@@ -1096,13 +1090,7 @@
     <t>result_qverkauf_flowsum</t>
   </si>
   <si>
-    <t>calc_einnahmen_qverkauf_schattenvariable</t>
-  </si>
-  <si>
     <t>calc_einnnahmen_qverkauf</t>
-  </si>
-  <si>
-    <t>Schattenvariable Einnahmen Wärmeverkauf</t>
   </si>
   <si>
     <t>Einnahmen aus Wärmeverkauf</t>
@@ -1633,41 +1621,38 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1677,6 +1662,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2094,7 +2082,7 @@
         <v>26</v>
       </c>
       <c r="E4" s="32">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="F4" s="28" t="s">
         <v>83</v>
@@ -2151,19 +2139,19 @@
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="59"/>
       <c r="B8" s="70" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C8" s="35" t="s">
         <v>84</v>
       </c>
       <c r="D8" s="35" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E8" s="36">
         <v>1.5</v>
       </c>
       <c r="F8" s="35" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -2173,7 +2161,7 @@
         <v>85</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="E9" s="31">
         <v>285.39999999999998</v>
@@ -2189,13 +2177,13 @@
         <v>10</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E10" s="31">
         <v>5110</v>
       </c>
       <c r="F10" s="31" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -2205,7 +2193,7 @@
         <v>11</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E11" s="33">
         <v>0.05</v>
@@ -2221,29 +2209,29 @@
         <v>86</v>
       </c>
       <c r="D12" s="28" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E12" s="31">
         <v>0.189</v>
       </c>
       <c r="F12" s="28" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="59"/>
       <c r="B13" s="67"/>
       <c r="C13" s="28" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D13" s="28" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E13" s="31">
         <v>1.375</v>
       </c>
       <c r="F13" s="28" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -2253,7 +2241,7 @@
         <v>13</v>
       </c>
       <c r="D14" s="28" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E14" s="34">
         <v>25</v>
@@ -2269,7 +2257,7 @@
         <v>15</v>
       </c>
       <c r="D15" s="37" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E15" s="38">
         <v>0.08</v>
@@ -2281,13 +2269,13 @@
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="59"/>
       <c r="B16" s="70" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C16" s="35" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="35" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="E16" s="39">
         <v>3.7</v>
@@ -2303,13 +2291,13 @@
         <v>84</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="E17" s="33">
         <v>0.27</v>
       </c>
       <c r="F17" s="28" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -2319,13 +2307,13 @@
         <v>10</v>
       </c>
       <c r="D18" s="28" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="E18" s="33">
         <v>700</v>
       </c>
       <c r="F18" s="28" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -2335,7 +2323,7 @@
         <v>11</v>
       </c>
       <c r="D19" s="28" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="E19" s="33">
         <v>0.02</v>
@@ -2351,7 +2339,7 @@
         <v>13</v>
       </c>
       <c r="D20" s="28" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E20" s="33">
         <v>20</v>
@@ -2367,7 +2355,7 @@
         <v>15</v>
       </c>
       <c r="D21" s="37" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E21" s="38">
         <v>0.05</v>
@@ -2379,35 +2367,35 @@
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="59"/>
       <c r="B22" s="63" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="C22" s="28" t="s">
         <v>84</v>
       </c>
       <c r="D22" s="28" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="E22" s="31">
         <v>0.2</v>
       </c>
       <c r="F22" s="28" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="59"/>
       <c r="B23" s="63"/>
       <c r="C23" s="28" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="E23" s="31">
         <v>0.92800000000000005</v>
       </c>
       <c r="F23" s="28" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -2417,23 +2405,23 @@
         <v>10</v>
       </c>
       <c r="D24" s="28" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="E24" s="31">
         <v>1640</v>
       </c>
       <c r="F24" s="28" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="59"/>
       <c r="B25" s="63"/>
       <c r="C25" s="28" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="D25" s="28" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="E25" s="33">
         <v>0.04</v>
@@ -2446,48 +2434,48 @@
       <c r="A26" s="59"/>
       <c r="B26" s="63"/>
       <c r="C26" s="28" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="D26" s="28" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="E26" s="33">
         <v>2.5</v>
       </c>
       <c r="F26" s="28" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="59"/>
       <c r="B27" s="63"/>
       <c r="C27" s="28" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="E27" s="33">
         <v>1.5</v>
       </c>
       <c r="F27" s="28" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="59"/>
       <c r="B28" s="63"/>
       <c r="C28" s="28" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="D28" s="28" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="E28" s="33">
         <v>1.5E-3</v>
       </c>
       <c r="F28" s="28" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
@@ -2497,7 +2485,7 @@
         <v>13</v>
       </c>
       <c r="D29" s="28" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="E29" s="34">
         <v>25</v>
@@ -2513,7 +2501,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="28" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="E30" s="33">
         <v>0.08</v>
@@ -2657,19 +2645,19 @@
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="59"/>
       <c r="B39" s="65" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="C39" s="29" t="s">
         <v>87</v>
       </c>
       <c r="D39" s="29" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="E39" s="40">
         <v>2.83</v>
       </c>
       <c r="F39" s="29" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
@@ -2679,7 +2667,7 @@
         <v>11</v>
       </c>
       <c r="D40" s="28" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="E40" s="33">
         <v>0.03</v>
@@ -2695,7 +2683,7 @@
         <v>13</v>
       </c>
       <c r="D41" s="28" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="E41" s="34">
         <v>30</v>
@@ -2711,7 +2699,7 @@
         <v>20</v>
       </c>
       <c r="D42" s="28" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="E42" s="33">
         <v>7.3999999999999999E-4</v>
@@ -2727,7 +2715,7 @@
         <v>35</v>
       </c>
       <c r="D43" s="28" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="E43" s="33">
         <v>0.98</v>
@@ -2743,7 +2731,7 @@
         <v>36</v>
       </c>
       <c r="D44" s="28" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="E44" s="33">
         <v>0.98</v>
@@ -2759,7 +2747,7 @@
         <v>15</v>
       </c>
       <c r="D45" s="28" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="E45" s="33">
         <v>0.05</v>
@@ -2775,7 +2763,7 @@
         <v>88</v>
       </c>
       <c r="D46" s="37" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="E46" s="38">
         <v>0</v>
@@ -2970,13 +2958,13 @@
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="61"/>
       <c r="B58" s="47" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="C58" s="48" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="D58" s="48" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="E58" s="49">
         <v>5</v>
@@ -2988,13 +2976,13 @@
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="61"/>
       <c r="B59" s="50" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="C59" s="51" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="D59" s="51" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="E59" s="52">
         <v>0</v>
@@ -3245,7 +3233,7 @@
         <v>78</v>
       </c>
       <c r="E74" s="46">
-        <v>-1E-4</v>
+        <v>0</v>
       </c>
       <c r="F74" s="45" t="s">
         <v>19</v>
@@ -3254,19 +3242,19 @@
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="59"/>
       <c r="B75" s="27" t="s">
+        <v>295</v>
+      </c>
+      <c r="C75" s="28" t="s">
+        <v>296</v>
+      </c>
+      <c r="D75" s="28" t="s">
         <v>297</v>
       </c>
-      <c r="C75" s="28" t="s">
-        <v>298</v>
-      </c>
-      <c r="D75" s="28" t="s">
-        <v>299</v>
-      </c>
       <c r="E75" s="33">
-        <v>-1E-4</v>
+        <v>0</v>
       </c>
       <c r="F75" s="28" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
@@ -3290,19 +3278,19 @@
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="60"/>
       <c r="B77" s="25" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C77" s="42" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D77" s="42" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="E77" s="43">
         <v>-0.6</v>
       </c>
       <c r="F77" s="42" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -3329,7 +3317,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AB2E79-6F94-41B5-A552-C40EC4890194}">
-  <dimension ref="A1:F151"/>
+  <dimension ref="A1:F149"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" style="5" customWidth="1"/>
@@ -3362,10 +3350,10 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="76" t="s">
+      <c r="A2" s="73" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="79" t="s">
+      <c r="B2" s="75" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="6" t="s">
@@ -3380,8 +3368,8 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="80"/>
-      <c r="B3" s="73"/>
+      <c r="A3" s="74"/>
+      <c r="B3" s="76"/>
       <c r="C3" s="5" t="s">
         <v>107</v>
       </c>
@@ -3394,8 +3382,8 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="80"/>
-      <c r="B4" s="73"/>
+      <c r="A4" s="74"/>
+      <c r="B4" s="76"/>
       <c r="C4" s="5" t="s">
         <v>84</v>
       </c>
@@ -3408,8 +3396,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="80"/>
-      <c r="B5" s="73"/>
+      <c r="A5" s="74"/>
+      <c r="B5" s="76"/>
       <c r="C5" s="5" t="s">
         <v>138</v>
       </c>
@@ -3422,8 +3410,8 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="80"/>
-      <c r="B6" s="73"/>
+      <c r="A6" s="74"/>
+      <c r="B6" s="76"/>
       <c r="C6" s="5" t="s">
         <v>141</v>
       </c>
@@ -3436,8 +3424,8 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="80"/>
-      <c r="B7" s="73"/>
+      <c r="A7" s="74"/>
+      <c r="B7" s="76"/>
       <c r="C7" s="5" t="s">
         <v>155</v>
       </c>
@@ -3450,8 +3438,8 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="80"/>
-      <c r="B8" s="73"/>
+      <c r="A8" s="74"/>
+      <c r="B8" s="76"/>
       <c r="C8" s="5" t="s">
         <v>196</v>
       </c>
@@ -3464,8 +3452,8 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="80"/>
-      <c r="B9" s="73"/>
+      <c r="A9" s="74"/>
+      <c r="B9" s="76"/>
       <c r="C9" s="5" t="s">
         <v>167</v>
       </c>
@@ -3478,8 +3466,8 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="80"/>
-      <c r="B10" s="73"/>
+      <c r="A10" s="74"/>
+      <c r="B10" s="76"/>
       <c r="C10" s="5" t="s">
         <v>188</v>
       </c>
@@ -3492,20 +3480,20 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="80"/>
-      <c r="B11" s="73"/>
+      <c r="A11" s="74"/>
+      <c r="B11" s="76"/>
       <c r="E11" s="10"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="80"/>
-      <c r="B12" s="72" t="s">
-        <v>229</v>
+      <c r="A12" s="74"/>
+      <c r="B12" s="77" t="s">
+        <v>227</v>
       </c>
       <c r="C12" s="12" t="s">
         <v>96</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E12" s="13"/>
       <c r="F12" s="12" t="s">
@@ -3513,27 +3501,27 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="80"/>
-      <c r="B13" s="73"/>
+      <c r="A13" s="74"/>
+      <c r="B13" s="76"/>
       <c r="C13" s="5" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="E13" s="8"/>
       <c r="F13" s="5" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="80"/>
-      <c r="B14" s="73"/>
+      <c r="A14" s="74"/>
+      <c r="B14" s="76"/>
       <c r="C14" s="5" t="s">
         <v>139</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E14" s="8"/>
       <c r="F14" s="8" t="s">
@@ -3541,27 +3529,27 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="80"/>
-      <c r="B15" s="73"/>
+      <c r="A15" s="74"/>
+      <c r="B15" s="76"/>
       <c r="C15" s="5" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="5" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="80"/>
-      <c r="B16" s="73"/>
+      <c r="A16" s="74"/>
+      <c r="B16" s="76"/>
       <c r="C16" s="5" t="s">
         <v>84</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E16" s="8"/>
       <c r="F16" s="5" t="s">
@@ -3569,13 +3557,13 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="80"/>
-      <c r="B17" s="73"/>
+      <c r="A17" s="74"/>
+      <c r="B17" s="76"/>
       <c r="C17" s="5" t="s">
         <v>141</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E17" s="8"/>
       <c r="F17" s="5" t="s">
@@ -3583,13 +3571,13 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="80"/>
-      <c r="B18" s="73"/>
+      <c r="A18" s="74"/>
+      <c r="B18" s="76"/>
       <c r="C18" s="5" t="s">
         <v>155</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E18" s="11"/>
       <c r="F18" s="5" t="s">
@@ -3597,13 +3585,13 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="80"/>
-      <c r="B19" s="73"/>
+      <c r="A19" s="74"/>
+      <c r="B19" s="76"/>
       <c r="C19" s="5" t="s">
         <v>196</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E19" s="11"/>
       <c r="F19" s="5" t="s">
@@ -3611,13 +3599,13 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="80"/>
-      <c r="B20" s="73"/>
+      <c r="A20" s="74"/>
+      <c r="B20" s="76"/>
       <c r="C20" s="5" t="s">
         <v>167</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E20" s="11"/>
       <c r="F20" s="5" t="s">
@@ -3625,13 +3613,13 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="80"/>
-      <c r="B21" s="73"/>
+      <c r="A21" s="74"/>
+      <c r="B21" s="76"/>
       <c r="C21" s="5" t="s">
         <v>188</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E21" s="11"/>
       <c r="F21" s="5" t="s">
@@ -3639,37 +3627,37 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="80"/>
-      <c r="B22" s="75"/>
+      <c r="A22" s="74"/>
+      <c r="B22" s="78"/>
       <c r="C22" s="14"/>
       <c r="D22" s="14"/>
       <c r="E22" s="15"/>
       <c r="F22" s="14"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="80"/>
-      <c r="B23" s="72" t="s">
-        <v>271</v>
+      <c r="A23" s="74"/>
+      <c r="B23" s="77" t="s">
+        <v>269</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>96</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E23" s="8"/>
       <c r="F23" s="5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="80"/>
-      <c r="B24" s="73"/>
+      <c r="A24" s="74"/>
+      <c r="B24" s="76"/>
       <c r="C24" s="5" t="s">
         <v>107</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="E24" s="8"/>
       <c r="F24" s="5" t="s">
@@ -3677,41 +3665,41 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="80"/>
-      <c r="B25" s="73"/>
+      <c r="A25" s="74"/>
+      <c r="B25" s="76"/>
       <c r="C25" s="5" t="s">
         <v>84</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E25" s="10"/>
       <c r="F25" s="5" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="80"/>
-      <c r="B26" s="73"/>
+      <c r="A26" s="74"/>
+      <c r="B26" s="76"/>
       <c r="C26" s="5" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="E26" s="11"/>
       <c r="F26" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="80"/>
-      <c r="B27" s="73"/>
+      <c r="A27" s="74"/>
+      <c r="B27" s="76"/>
       <c r="C27" s="5" t="s">
         <v>141</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="E27" s="11"/>
       <c r="F27" s="5" t="s">
@@ -3719,13 +3707,13 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="80"/>
-      <c r="B28" s="73"/>
+      <c r="A28" s="74"/>
+      <c r="B28" s="76"/>
       <c r="C28" s="5" t="s">
         <v>155</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="E28" s="11"/>
       <c r="F28" s="5" t="s">
@@ -3733,13 +3721,13 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="80"/>
-      <c r="B29" s="73"/>
+      <c r="A29" s="74"/>
+      <c r="B29" s="76"/>
       <c r="C29" s="5" t="s">
         <v>196</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="E29" s="11"/>
       <c r="F29" s="5" t="s">
@@ -3747,13 +3735,13 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="80"/>
-      <c r="B30" s="73"/>
+      <c r="A30" s="74"/>
+      <c r="B30" s="76"/>
       <c r="C30" s="5" t="s">
         <v>167</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E30" s="10"/>
       <c r="F30" s="5" t="s">
@@ -3761,13 +3749,13 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="80"/>
-      <c r="B31" s="73"/>
+      <c r="A31" s="74"/>
+      <c r="B31" s="76"/>
       <c r="C31" s="5" t="s">
         <v>188</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="E31" s="10"/>
       <c r="F31" s="5" t="s">
@@ -3775,23 +3763,23 @@
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="80"/>
-      <c r="B32" s="75"/>
+      <c r="A32" s="74"/>
+      <c r="B32" s="78"/>
       <c r="C32" s="14"/>
       <c r="D32" s="14"/>
       <c r="E32" s="15"/>
       <c r="F32" s="14"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="80"/>
-      <c r="B33" s="82" t="s">
-        <v>358</v>
+      <c r="A33" s="74"/>
+      <c r="B33" s="79" t="s">
+        <v>354</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>96</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="E33" s="8"/>
       <c r="F33" s="5" t="s">
@@ -3799,13 +3787,13 @@
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="80"/>
-      <c r="B34" s="82"/>
+      <c r="A34" s="74"/>
+      <c r="B34" s="79"/>
       <c r="C34" s="5" t="s">
         <v>107</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="E34" s="8"/>
       <c r="F34" s="5" t="s">
@@ -3813,13 +3801,13 @@
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="80"/>
-      <c r="B35" s="82"/>
+      <c r="A35" s="74"/>
+      <c r="B35" s="79"/>
       <c r="C35" s="5" t="s">
         <v>84</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="E35" s="10"/>
       <c r="F35" s="5" t="s">
@@ -3827,55 +3815,55 @@
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="80"/>
-      <c r="B36" s="82"/>
+      <c r="A36" s="74"/>
+      <c r="B36" s="79"/>
       <c r="C36" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="E36" s="10"/>
       <c r="F36" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="80"/>
-      <c r="B37" s="82"/>
+      <c r="A37" s="74"/>
+      <c r="B37" s="79"/>
       <c r="C37" s="5" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="E37" s="10"/>
       <c r="F37" s="5" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="80"/>
-      <c r="B38" s="82"/>
+      <c r="A38" s="74"/>
+      <c r="B38" s="79"/>
       <c r="C38" s="5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="E38" s="11"/>
       <c r="F38" s="5" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="80"/>
-      <c r="B39" s="82"/>
+      <c r="A39" s="74"/>
+      <c r="B39" s="79"/>
       <c r="C39" s="5" t="s">
         <v>141</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="E39" s="11"/>
       <c r="F39" s="5" t="s">
@@ -3883,13 +3871,13 @@
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="80"/>
-      <c r="B40" s="82"/>
+      <c r="A40" s="74"/>
+      <c r="B40" s="79"/>
       <c r="C40" s="5" t="s">
         <v>155</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="E40" s="11"/>
       <c r="F40" s="5" t="s">
@@ -3897,13 +3885,13 @@
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="80"/>
-      <c r="B41" s="82"/>
+      <c r="A41" s="74"/>
+      <c r="B41" s="79"/>
       <c r="C41" s="5" t="s">
         <v>161</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="E41" s="11"/>
       <c r="F41" s="5" t="s">
@@ -3911,13 +3899,13 @@
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="80"/>
-      <c r="B42" s="82"/>
+      <c r="A42" s="74"/>
+      <c r="B42" s="79"/>
       <c r="C42" s="5" t="s">
         <v>196</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="E42" s="11"/>
       <c r="F42" s="5" t="s">
@@ -3925,13 +3913,13 @@
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="80"/>
-      <c r="B43" s="82"/>
+      <c r="A43" s="74"/>
+      <c r="B43" s="79"/>
       <c r="C43" s="5" t="s">
         <v>167</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="E43" s="10"/>
       <c r="F43" s="5" t="s">
@@ -3939,13 +3927,13 @@
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="80"/>
-      <c r="B44" s="82"/>
+      <c r="A44" s="74"/>
+      <c r="B44" s="79"/>
       <c r="C44" s="5" t="s">
         <v>188</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="E44" s="10"/>
       <c r="F44" s="5" t="s">
@@ -3953,15 +3941,15 @@
       </c>
     </row>
     <row r="45" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="80"/>
-      <c r="B45" s="82"/>
+      <c r="A45" s="74"/>
+      <c r="B45" s="79"/>
       <c r="E45" s="10"/>
     </row>
     <row r="46" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="76" t="s">
+      <c r="A46" s="73" t="s">
         <v>71</v>
       </c>
-      <c r="B46" s="84" t="s">
+      <c r="B46" s="83" t="s">
         <v>3</v>
       </c>
       <c r="C46" s="6" t="s">
@@ -3972,12 +3960,12 @@
       </c>
       <c r="E46" s="16"/>
       <c r="F46" s="6" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="80"/>
-      <c r="B47" s="82"/>
+      <c r="A47" s="74"/>
+      <c r="B47" s="79"/>
       <c r="C47" s="5" t="s">
         <v>111</v>
       </c>
@@ -3986,12 +3974,12 @@
       </c>
       <c r="E47" s="10"/>
       <c r="F47" s="5" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="80"/>
-      <c r="B48" s="82"/>
+      <c r="A48" s="74"/>
+      <c r="B48" s="79"/>
       <c r="C48" s="5" t="s">
         <v>135</v>
       </c>
@@ -4004,8 +3992,8 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="80"/>
-      <c r="B49" s="82"/>
+      <c r="A49" s="74"/>
+      <c r="B49" s="79"/>
       <c r="C49" s="5" t="s">
         <v>136</v>
       </c>
@@ -4018,8 +4006,8 @@
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="80"/>
-      <c r="B50" s="82"/>
+      <c r="A50" s="74"/>
+      <c r="B50" s="79"/>
       <c r="C50" s="5" t="s">
         <v>141</v>
       </c>
@@ -4032,8 +4020,8 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="80"/>
-      <c r="B51" s="82"/>
+      <c r="A51" s="74"/>
+      <c r="B51" s="79"/>
       <c r="C51" s="5" t="s">
         <v>155</v>
       </c>
@@ -4046,8 +4034,8 @@
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="80"/>
-      <c r="B52" s="82"/>
+      <c r="A52" s="74"/>
+      <c r="B52" s="79"/>
       <c r="C52" s="5" t="s">
         <v>196</v>
       </c>
@@ -4060,8 +4048,8 @@
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="80"/>
-      <c r="B53" s="82"/>
+      <c r="A53" s="74"/>
+      <c r="B53" s="79"/>
       <c r="C53" s="5" t="s">
         <v>167</v>
       </c>
@@ -4074,8 +4062,8 @@
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="80"/>
-      <c r="B54" s="82"/>
+      <c r="A54" s="74"/>
+      <c r="B54" s="79"/>
       <c r="C54" s="5" t="s">
         <v>188</v>
       </c>
@@ -4088,79 +4076,79 @@
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="80"/>
-      <c r="B55" s="85"/>
+      <c r="A55" s="74"/>
+      <c r="B55" s="84"/>
       <c r="C55" s="14"/>
       <c r="D55" s="14"/>
       <c r="E55" s="15"/>
       <c r="F55" s="14"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="80"/>
-      <c r="B56" s="82" t="s">
-        <v>315</v>
+      <c r="A56" s="74"/>
+      <c r="B56" s="79" t="s">
+        <v>311</v>
       </c>
       <c r="C56" s="5" t="s">
         <v>113</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="E56" s="8"/>
       <c r="F56" s="5" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="80"/>
-      <c r="B57" s="82"/>
+      <c r="A57" s="74"/>
+      <c r="B57" s="79"/>
       <c r="C57" s="5" t="s">
         <v>111</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="E57" s="10"/>
       <c r="F57" s="5" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="80"/>
-      <c r="B58" s="82"/>
+      <c r="A58" s="74"/>
+      <c r="B58" s="79"/>
       <c r="C58" s="5" t="s">
         <v>135</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="E58" s="11"/>
       <c r="F58" s="5" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="80"/>
-      <c r="B59" s="82"/>
+      <c r="A59" s="74"/>
+      <c r="B59" s="79"/>
       <c r="C59" s="5" t="s">
         <v>136</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="E59" s="10"/>
       <c r="F59" s="5" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="80"/>
-      <c r="B60" s="82"/>
+      <c r="A60" s="74"/>
+      <c r="B60" s="79"/>
       <c r="C60" s="5" t="s">
         <v>141</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="E60" s="10"/>
       <c r="F60" s="5" t="s">
@@ -4168,13 +4156,13 @@
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="80"/>
-      <c r="B61" s="82"/>
+      <c r="A61" s="74"/>
+      <c r="B61" s="79"/>
       <c r="C61" s="5" t="s">
         <v>155</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="E61" s="10"/>
       <c r="F61" s="5" t="s">
@@ -4182,13 +4170,13 @@
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="80"/>
-      <c r="B62" s="82"/>
+      <c r="A62" s="74"/>
+      <c r="B62" s="79"/>
       <c r="C62" s="5" t="s">
         <v>196</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="E62" s="10"/>
       <c r="F62" s="5" t="s">
@@ -4196,13 +4184,13 @@
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="80"/>
-      <c r="B63" s="82"/>
+      <c r="A63" s="74"/>
+      <c r="B63" s="79"/>
       <c r="C63" s="5" t="s">
         <v>167</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="E63" s="10"/>
       <c r="F63" s="5" t="s">
@@ -4210,13 +4198,13 @@
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="80"/>
-      <c r="B64" s="82"/>
+      <c r="A64" s="74"/>
+      <c r="B64" s="79"/>
       <c r="C64" s="5" t="s">
         <v>188</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="E64" s="10"/>
       <c r="F64" s="5" t="s">
@@ -4224,13 +4212,13 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="80"/>
-      <c r="B65" s="85"/>
+      <c r="A65" s="74"/>
+      <c r="B65" s="84"/>
       <c r="E65" s="10"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="80"/>
-      <c r="B66" s="83" t="s">
+      <c r="A66" s="74"/>
+      <c r="B66" s="81" t="s">
         <v>6</v>
       </c>
       <c r="C66" s="12" t="s">
@@ -4245,8 +4233,8 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="80"/>
-      <c r="B67" s="82"/>
+      <c r="A67" s="74"/>
+      <c r="B67" s="79"/>
       <c r="C67" s="5" t="s">
         <v>113</v>
       </c>
@@ -4259,8 +4247,8 @@
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="80"/>
-      <c r="B68" s="73"/>
+      <c r="A68" s="74"/>
+      <c r="B68" s="76"/>
       <c r="C68" s="5" t="s">
         <v>111</v>
       </c>
@@ -4273,8 +4261,8 @@
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="80"/>
-      <c r="B69" s="73"/>
+      <c r="A69" s="74"/>
+      <c r="B69" s="76"/>
       <c r="C69" s="5" t="s">
         <v>107</v>
       </c>
@@ -4287,8 +4275,8 @@
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="80"/>
-      <c r="B70" s="73"/>
+      <c r="A70" s="74"/>
+      <c r="B70" s="76"/>
       <c r="C70" s="5" t="s">
         <v>126</v>
       </c>
@@ -4301,8 +4289,8 @@
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="80"/>
-      <c r="B71" s="73"/>
+      <c r="A71" s="74"/>
+      <c r="B71" s="76"/>
       <c r="C71" s="5" t="s">
         <v>127</v>
       </c>
@@ -4315,8 +4303,8 @@
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="80"/>
-      <c r="B72" s="73"/>
+      <c r="A72" s="74"/>
+      <c r="B72" s="76"/>
       <c r="C72" s="5" t="s">
         <v>141</v>
       </c>
@@ -4329,8 +4317,8 @@
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="80"/>
-      <c r="B73" s="73"/>
+      <c r="A73" s="74"/>
+      <c r="B73" s="76"/>
       <c r="C73" s="5" t="s">
         <v>155</v>
       </c>
@@ -4343,8 +4331,8 @@
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="80"/>
-      <c r="B74" s="73"/>
+      <c r="A74" s="74"/>
+      <c r="B74" s="76"/>
       <c r="C74" s="5" t="s">
         <v>196</v>
       </c>
@@ -4357,8 +4345,8 @@
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="80"/>
-      <c r="B75" s="73"/>
+      <c r="A75" s="74"/>
+      <c r="B75" s="76"/>
       <c r="C75" s="5" t="s">
         <v>167</v>
       </c>
@@ -4371,8 +4359,8 @@
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76" s="80"/>
-      <c r="B76" s="73"/>
+      <c r="A76" s="74"/>
+      <c r="B76" s="76"/>
       <c r="C76" s="5" t="s">
         <v>188</v>
       </c>
@@ -4385,18 +4373,18 @@
       </c>
     </row>
     <row r="77" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="81"/>
-      <c r="B77" s="78"/>
+      <c r="A77" s="80"/>
+      <c r="B77" s="82"/>
       <c r="C77" s="18"/>
       <c r="D77" s="18"/>
       <c r="E77" s="19"/>
       <c r="F77" s="18"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="76" t="s">
+      <c r="A78" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="B78" s="79" t="s">
+      <c r="B78" s="75" t="s">
         <v>73</v>
       </c>
       <c r="C78" s="6" t="s">
@@ -4411,8 +4399,8 @@
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="80"/>
-      <c r="B79" s="74"/>
+      <c r="A79" s="74"/>
+      <c r="B79" s="72"/>
       <c r="C79" s="20" t="s">
         <v>153</v>
       </c>
@@ -4425,37 +4413,37 @@
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80" s="80"/>
-      <c r="B80" s="75"/>
+      <c r="A80" s="74"/>
+      <c r="B80" s="78"/>
       <c r="C80" s="14"/>
       <c r="D80" s="14"/>
       <c r="E80" s="22"/>
       <c r="F80" s="14"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81" s="80"/>
-      <c r="B81" s="72" t="s">
-        <v>341</v>
+      <c r="A81" s="74"/>
+      <c r="B81" s="77" t="s">
+        <v>337</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="D81" s="12" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="E81" s="13"/>
       <c r="F81" s="12" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" s="80"/>
-      <c r="B82" s="74"/>
+      <c r="A82" s="74"/>
+      <c r="B82" s="72"/>
       <c r="C82" s="20" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="D82" s="20" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="E82" s="21"/>
       <c r="F82" s="20" t="s">
@@ -4463,23 +4451,23 @@
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="80"/>
-      <c r="B83" s="75"/>
+      <c r="A83" s="74"/>
+      <c r="B83" s="78"/>
       <c r="C83" s="14"/>
       <c r="D83" s="14"/>
       <c r="E83" s="22"/>
       <c r="F83" s="14"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" s="80"/>
-      <c r="B84" s="74" t="s">
-        <v>383</v>
+      <c r="A84" s="74"/>
+      <c r="B84" s="72" t="s">
+        <v>379</v>
       </c>
       <c r="C84" s="20" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="D84" s="20" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="E84" s="21"/>
       <c r="F84" s="20" t="s">
@@ -4487,13 +4475,13 @@
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" s="80"/>
-      <c r="B85" s="74"/>
+      <c r="A85" s="74"/>
+      <c r="B85" s="72"/>
       <c r="C85" s="5" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="E85" s="8"/>
       <c r="F85" s="5" t="s">
@@ -4501,13 +4489,13 @@
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" s="80"/>
-      <c r="B86" s="74"/>
+      <c r="A86" s="74"/>
+      <c r="B86" s="72"/>
       <c r="E86" s="8"/>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A87" s="80"/>
-      <c r="B87" s="83" t="s">
+      <c r="A87" s="74"/>
+      <c r="B87" s="81" t="s">
         <v>4</v>
       </c>
       <c r="C87" s="12" t="s">
@@ -4522,8 +4510,8 @@
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A88" s="80"/>
-      <c r="B88" s="82"/>
+      <c r="A88" s="74"/>
+      <c r="B88" s="79"/>
       <c r="C88" s="5" t="s">
         <v>107</v>
       </c>
@@ -4536,8 +4524,8 @@
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" s="80"/>
-      <c r="B89" s="82"/>
+      <c r="A89" s="74"/>
+      <c r="B89" s="79"/>
       <c r="C89" s="5" t="s">
         <v>122</v>
       </c>
@@ -4550,8 +4538,8 @@
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" s="80"/>
-      <c r="B90" s="82"/>
+      <c r="A90" s="74"/>
+      <c r="B90" s="79"/>
       <c r="C90" s="5" t="s">
         <v>141</v>
       </c>
@@ -4564,8 +4552,8 @@
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" s="80"/>
-      <c r="B91" s="82"/>
+      <c r="A91" s="74"/>
+      <c r="B91" s="79"/>
       <c r="C91" s="5" t="s">
         <v>155</v>
       </c>
@@ -4578,8 +4566,8 @@
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" s="80"/>
-      <c r="B92" s="82"/>
+      <c r="A92" s="74"/>
+      <c r="B92" s="79"/>
       <c r="C92" s="5" t="s">
         <v>161</v>
       </c>
@@ -4592,8 +4580,8 @@
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" s="80"/>
-      <c r="B93" s="82"/>
+      <c r="A93" s="74"/>
+      <c r="B93" s="79"/>
       <c r="C93" s="5" t="s">
         <v>196</v>
       </c>
@@ -4606,8 +4594,8 @@
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" s="80"/>
-      <c r="B94" s="82"/>
+      <c r="A94" s="74"/>
+      <c r="B94" s="79"/>
       <c r="C94" s="5" t="s">
         <v>167</v>
       </c>
@@ -4620,8 +4608,8 @@
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" s="80"/>
-      <c r="B95" s="82"/>
+      <c r="A95" s="74"/>
+      <c r="B95" s="79"/>
       <c r="C95" s="5" t="s">
         <v>188</v>
       </c>
@@ -4634,12 +4622,12 @@
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" s="80"/>
-      <c r="B96" s="85"/>
+      <c r="A96" s="74"/>
+      <c r="B96" s="84"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A97" s="80"/>
-      <c r="B97" s="83" t="s">
+      <c r="A97" s="74"/>
+      <c r="B97" s="81" t="s">
         <v>5</v>
       </c>
       <c r="C97" s="12" t="s">
@@ -4654,8 +4642,8 @@
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A98" s="80"/>
-      <c r="B98" s="82"/>
+      <c r="A98" s="74"/>
+      <c r="B98" s="79"/>
       <c r="C98" s="5" t="s">
         <v>108</v>
       </c>
@@ -4668,8 +4656,8 @@
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A99" s="80"/>
-      <c r="B99" s="82"/>
+      <c r="A99" s="74"/>
+      <c r="B99" s="79"/>
       <c r="C99" s="5" t="s">
         <v>120</v>
       </c>
@@ -4682,8 +4670,8 @@
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" s="80"/>
-      <c r="B100" s="82"/>
+      <c r="A100" s="74"/>
+      <c r="B100" s="79"/>
       <c r="C100" s="5" t="s">
         <v>141</v>
       </c>
@@ -4696,8 +4684,8 @@
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" s="80"/>
-      <c r="B101" s="82"/>
+      <c r="A101" s="74"/>
+      <c r="B101" s="79"/>
       <c r="C101" s="5" t="s">
         <v>155</v>
       </c>
@@ -4710,8 +4698,8 @@
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" s="80"/>
-      <c r="B102" s="82"/>
+      <c r="A102" s="74"/>
+      <c r="B102" s="79"/>
       <c r="C102" s="5" t="s">
         <v>161</v>
       </c>
@@ -4724,8 +4712,8 @@
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" s="80"/>
-      <c r="B103" s="82"/>
+      <c r="A103" s="74"/>
+      <c r="B103" s="79"/>
       <c r="C103" s="5" t="s">
         <v>196</v>
       </c>
@@ -4738,8 +4726,8 @@
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" s="80"/>
-      <c r="B104" s="82"/>
+      <c r="A104" s="74"/>
+      <c r="B104" s="79"/>
       <c r="C104" s="5" t="s">
         <v>167</v>
       </c>
@@ -4752,8 +4740,8 @@
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" s="80"/>
-      <c r="B105" s="82"/>
+      <c r="A105" s="74"/>
+      <c r="B105" s="79"/>
       <c r="C105" s="5" t="s">
         <v>188</v>
       </c>
@@ -4766,14 +4754,14 @@
       </c>
     </row>
     <row r="106" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A106" s="81"/>
-      <c r="B106" s="86"/>
+      <c r="A106" s="80"/>
+      <c r="B106" s="85"/>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" s="76" t="s">
+      <c r="A107" s="73" t="s">
         <v>76</v>
       </c>
-      <c r="B107" s="79" t="s">
+      <c r="B107" s="75" t="s">
         <v>73</v>
       </c>
       <c r="C107" s="6" t="s">
@@ -4788,13 +4776,13 @@
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" s="80"/>
-      <c r="B108" s="73"/>
+      <c r="A108" s="74"/>
+      <c r="B108" s="76"/>
       <c r="C108" s="5" t="s">
-        <v>228</v>
+        <v>150</v>
       </c>
       <c r="D108" s="5" t="s">
-        <v>227</v>
+        <v>147</v>
       </c>
       <c r="E108" s="10"/>
       <c r="F108" s="5" t="s">
@@ -4802,541 +4790,524 @@
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A109" s="80"/>
-      <c r="B109" s="73"/>
-      <c r="C109" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="D109" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="E109" s="10"/>
-      <c r="F109" s="5" t="s">
-        <v>149</v>
-      </c>
+      <c r="A109" s="74"/>
+      <c r="B109" s="78"/>
+      <c r="C109" s="14"/>
+      <c r="D109" s="14"/>
+      <c r="E109" s="15"/>
+      <c r="F109" s="14"/>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A110" s="80"/>
-      <c r="B110" s="75"/>
-      <c r="C110" s="14"/>
-      <c r="D110" s="14"/>
-      <c r="E110" s="15"/>
-      <c r="F110" s="14"/>
+      <c r="A110" s="74"/>
+      <c r="B110" s="77" t="s">
+        <v>299</v>
+      </c>
+      <c r="C110" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D110" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="E110" s="10"/>
+      <c r="F110" s="5" t="s">
+        <v>290</v>
+      </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A111" s="80"/>
-      <c r="B111" s="72" t="s">
-        <v>301</v>
-      </c>
+      <c r="A111" s="74"/>
+      <c r="B111" s="76"/>
       <c r="C111" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="D111" s="5" t="s">
         <v>302</v>
-      </c>
-      <c r="D111" s="5" t="s">
-        <v>303</v>
       </c>
       <c r="E111" s="10"/>
       <c r="F111" s="5" t="s">
-        <v>292</v>
+        <v>149</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A112" s="80"/>
-      <c r="B112" s="73"/>
-      <c r="C112" s="5" t="s">
-        <v>306</v>
-      </c>
-      <c r="D112" s="5" t="s">
-        <v>304</v>
-      </c>
+      <c r="A112" s="74"/>
+      <c r="B112" s="78"/>
       <c r="E112" s="10"/>
-      <c r="F112" s="5" t="s">
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A113" s="74"/>
+      <c r="B113" s="77" t="s">
+        <v>79</v>
+      </c>
+      <c r="C113" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="D113" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="E113" s="17"/>
+      <c r="F113" s="12" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A114" s="74"/>
+      <c r="B114" s="76"/>
+      <c r="C114" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="E114" s="10"/>
+      <c r="F114" s="5" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A113" s="80"/>
-      <c r="B113" s="73"/>
-      <c r="C113" s="5" t="s">
-        <v>307</v>
-      </c>
-      <c r="D113" s="5" t="s">
-        <v>305</v>
-      </c>
-      <c r="E113" s="10"/>
-      <c r="F113" s="5" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A114" s="80"/>
-      <c r="B114" s="75"/>
-      <c r="E114" s="10"/>
-    </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A115" s="80"/>
-      <c r="B115" s="72" t="s">
-        <v>79</v>
-      </c>
-      <c r="C115" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="D115" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="E115" s="17"/>
-      <c r="F115" s="12" t="s">
-        <v>132</v>
-      </c>
+      <c r="A115" s="74"/>
+      <c r="B115" s="78"/>
+      <c r="C115" s="14"/>
+      <c r="D115" s="14"/>
+      <c r="E115" s="15"/>
+      <c r="F115" s="14"/>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A116" s="80"/>
-      <c r="B116" s="73"/>
+      <c r="A116" s="74"/>
+      <c r="B116" s="77" t="s">
+        <v>258</v>
+      </c>
       <c r="C116" s="5" t="s">
-        <v>151</v>
+        <v>257</v>
       </c>
       <c r="D116" s="5" t="s">
-        <v>148</v>
+        <v>260</v>
       </c>
       <c r="E116" s="10"/>
       <c r="F116" s="5" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A117" s="74"/>
+      <c r="B117" s="76"/>
+      <c r="C117" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="D117" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="E117" s="10"/>
+      <c r="F117" s="5" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A117" s="80"/>
-      <c r="B117" s="75"/>
-      <c r="C117" s="14"/>
-      <c r="D117" s="14"/>
-      <c r="E117" s="15"/>
-      <c r="F117" s="14"/>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A118" s="80"/>
-      <c r="B118" s="72" t="s">
-        <v>260</v>
-      </c>
-      <c r="C118" s="5" t="s">
-        <v>259</v>
-      </c>
-      <c r="D118" s="5" t="s">
-        <v>262</v>
-      </c>
-      <c r="E118" s="10"/>
-      <c r="F118" s="5" t="s">
-        <v>256</v>
-      </c>
+      <c r="B118" s="82"/>
+      <c r="C118" s="18"/>
+      <c r="D118" s="18"/>
+      <c r="E118" s="19"/>
+      <c r="F118" s="18"/>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A119" s="80"/>
-      <c r="B119" s="73"/>
-      <c r="C119" s="5" t="s">
-        <v>261</v>
-      </c>
-      <c r="D119" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="E119" s="10"/>
-      <c r="F119" s="5" t="s">
+      <c r="A119" s="73" t="s">
+        <v>163</v>
+      </c>
+      <c r="B119" s="75" t="s">
+        <v>13</v>
+      </c>
+      <c r="C119" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D119" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="E119" s="6"/>
+      <c r="F119" s="6" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A120" s="86"/>
+      <c r="B120" s="76"/>
+      <c r="C120" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D120" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="F120" s="5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A121" s="86"/>
+      <c r="B121" s="78"/>
+      <c r="C121" s="14"/>
+      <c r="D121" s="14"/>
+      <c r="E121" s="14"/>
+      <c r="F121" s="14"/>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A122" s="86"/>
+      <c r="B122" s="77" t="s">
+        <v>183</v>
+      </c>
+      <c r="C122" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="D122" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="F122" s="5" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="120" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A120" s="81"/>
-      <c r="B120" s="78"/>
-      <c r="C120" s="18"/>
-      <c r="D120" s="18"/>
-      <c r="E120" s="19"/>
-      <c r="F120" s="18"/>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A121" s="76" t="s">
-        <v>163</v>
-      </c>
-      <c r="B121" s="79" t="s">
-        <v>13</v>
-      </c>
-      <c r="C121" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D121" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="E121" s="6"/>
-      <c r="F121" s="6" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A122" s="77"/>
-      <c r="B122" s="73"/>
-      <c r="C122" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="D122" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="F122" s="5" t="s">
-        <v>140</v>
-      </c>
-    </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A123" s="77"/>
-      <c r="B123" s="75"/>
-      <c r="C123" s="14"/>
-      <c r="D123" s="14"/>
-      <c r="E123" s="14"/>
-      <c r="F123" s="14"/>
+      <c r="A123" s="86"/>
+      <c r="B123" s="76"/>
+      <c r="C123" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="D123" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="F123" s="5" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A124" s="77"/>
-      <c r="B124" s="72" t="s">
-        <v>183</v>
-      </c>
+      <c r="A124" s="86"/>
+      <c r="B124" s="76"/>
       <c r="C124" s="5" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="D124" s="5" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="F124" s="5" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A125" s="77"/>
-      <c r="B125" s="73"/>
+      <c r="A125" s="86"/>
+      <c r="B125" s="76"/>
       <c r="C125" s="5" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D125" s="5" t="s">
-        <v>309</v>
+        <v>178</v>
       </c>
       <c r="F125" s="5" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A126" s="77"/>
-      <c r="B126" s="73"/>
+      <c r="A126" s="86"/>
+      <c r="B126" s="76"/>
       <c r="C126" s="5" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="D126" s="5" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="F126" s="5" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A127" s="77"/>
-      <c r="B127" s="73"/>
+      <c r="A127" s="86"/>
+      <c r="B127" s="76"/>
       <c r="C127" s="5" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="D127" s="5" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="F127" s="5" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A128" s="77"/>
-      <c r="B128" s="73"/>
-      <c r="C128" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="D128" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="F128" s="5" t="s">
-        <v>149</v>
-      </c>
+      <c r="A128" s="86"/>
+      <c r="B128" s="76"/>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A129" s="77"/>
-      <c r="B129" s="73"/>
-      <c r="C129" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="D129" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="F129" s="5" t="s">
-        <v>149</v>
+      <c r="A129" s="86"/>
+      <c r="B129" s="77" t="s">
+        <v>206</v>
+      </c>
+      <c r="C129" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="D129" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="E129" s="12"/>
+      <c r="F129" s="12" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A130" s="77"/>
-      <c r="B130" s="73"/>
+      <c r="A130" s="86"/>
+      <c r="B130" s="76"/>
+      <c r="C130" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="F130" s="5" t="s">
+        <v>208</v>
+      </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A131" s="77"/>
-      <c r="B131" s="72" t="s">
-        <v>206</v>
-      </c>
-      <c r="C131" s="12" t="s">
-        <v>203</v>
-      </c>
-      <c r="D131" s="12" t="s">
-        <v>207</v>
-      </c>
-      <c r="E131" s="12"/>
-      <c r="F131" s="12" t="s">
-        <v>208</v>
+      <c r="A131" s="86"/>
+      <c r="B131" s="76"/>
+      <c r="C131" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D131" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="F131" s="5" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A132" s="77"/>
-      <c r="B132" s="73"/>
+      <c r="A132" s="86"/>
+      <c r="B132" s="76"/>
       <c r="C132" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D132" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F132" s="5" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A133" s="77"/>
-      <c r="B133" s="73"/>
+      <c r="A133" s="86"/>
+      <c r="B133" s="76"/>
       <c r="C133" s="5" t="s">
-        <v>215</v>
+        <v>306</v>
       </c>
       <c r="D133" s="5" t="s">
-        <v>214</v>
+        <v>307</v>
       </c>
       <c r="F133" s="5" t="s">
-        <v>219</v>
+        <v>310</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A134" s="77"/>
-      <c r="B134" s="73"/>
+      <c r="A134" s="86"/>
+      <c r="B134" s="76"/>
       <c r="C134" s="5" t="s">
-        <v>205</v>
+        <v>330</v>
       </c>
       <c r="D134" s="5" t="s">
-        <v>209</v>
+        <v>331</v>
       </c>
       <c r="F134" s="5" t="s">
-        <v>208</v>
+        <v>310</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A135" s="77"/>
-      <c r="B135" s="73"/>
+      <c r="A135" s="86"/>
+      <c r="B135" s="76"/>
       <c r="C135" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="D135" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="F135" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="D135" s="5" t="s">
-        <v>311</v>
-      </c>
-      <c r="F135" s="5" t="s">
-        <v>314</v>
-      </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A136" s="77"/>
-      <c r="B136" s="73"/>
+      <c r="A136" s="86"/>
+      <c r="B136" s="76"/>
       <c r="C136" s="5" t="s">
-        <v>334</v>
+        <v>217</v>
       </c>
       <c r="D136" s="5" t="s">
-        <v>335</v>
+        <v>216</v>
       </c>
       <c r="F136" s="5" t="s">
-        <v>314</v>
+        <v>218</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A137" s="77"/>
-      <c r="B137" s="73"/>
+      <c r="A137" s="86"/>
+      <c r="B137" s="76"/>
       <c r="C137" s="5" t="s">
-        <v>336</v>
+        <v>221</v>
       </c>
       <c r="D137" s="5" t="s">
-        <v>337</v>
+        <v>211</v>
       </c>
       <c r="F137" s="5" t="s">
-        <v>314</v>
+        <v>212</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A138" s="77"/>
-      <c r="B138" s="73"/>
+      <c r="A138" s="86"/>
+      <c r="B138" s="76"/>
       <c r="C138" s="5" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="D138" s="5" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="F138" s="5" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A139" s="77"/>
-      <c r="B139" s="73"/>
+      <c r="A139" s="86"/>
+      <c r="B139" s="76"/>
       <c r="C139" s="5" t="s">
-        <v>221</v>
+        <v>262</v>
       </c>
       <c r="D139" s="5" t="s">
-        <v>211</v>
+        <v>365</v>
       </c>
       <c r="F139" s="5" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A140" s="77"/>
-      <c r="B140" s="73"/>
+      <c r="A140" s="86"/>
+      <c r="B140" s="76"/>
       <c r="C140" s="5" t="s">
-        <v>202</v>
+        <v>264</v>
       </c>
       <c r="D140" s="5" t="s">
-        <v>220</v>
+        <v>263</v>
       </c>
       <c r="F140" s="5" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A141" s="86"/>
+      <c r="B141" s="76"/>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A142" s="86"/>
+      <c r="B142" s="77" t="s">
+        <v>222</v>
+      </c>
+      <c r="C142" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="D142" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="E142" s="12"/>
+      <c r="F142" s="12" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A143" s="86"/>
+      <c r="B143" s="72"/>
+      <c r="C143" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="D143" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="F143" s="5" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A144" s="86"/>
+      <c r="B144" s="72"/>
+      <c r="C144" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="D144" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="F144" s="5" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A141" s="77"/>
-      <c r="B141" s="73"/>
-      <c r="C141" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="D141" s="5" t="s">
-        <v>369</v>
-      </c>
-      <c r="F141" s="5" t="s">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A145" s="86"/>
+      <c r="B145" s="72"/>
+      <c r="C145" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="D145" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F145" s="5" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A142" s="77"/>
-      <c r="B142" s="73"/>
-      <c r="C142" s="5" t="s">
-        <v>266</v>
-      </c>
-      <c r="D142" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="F142" s="5" t="s">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A146" s="86"/>
+      <c r="B146" s="72"/>
+      <c r="C146" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="D146" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="F146" s="5" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A143" s="77"/>
-      <c r="B143" s="73"/>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A144" s="77"/>
-      <c r="B144" s="72" t="s">
-        <v>222</v>
-      </c>
-      <c r="C144" s="12" t="s">
-        <v>224</v>
-      </c>
-      <c r="D144" s="12" t="s">
-        <v>223</v>
-      </c>
-      <c r="E144" s="12"/>
-      <c r="F144" s="12" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A145" s="77"/>
-      <c r="B145" s="74"/>
-      <c r="C145" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="D145" s="5" t="s">
-        <v>313</v>
-      </c>
-      <c r="F145" s="5" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A146" s="77"/>
-      <c r="B146" s="74"/>
-      <c r="C146" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="D146" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="F146" s="5" t="s">
-        <v>212</v>
-      </c>
-    </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A147" s="77"/>
-      <c r="B147" s="74"/>
-      <c r="C147" s="5" t="s">
-        <v>267</v>
-      </c>
-      <c r="D147" s="5" t="s">
-        <v>268</v>
-      </c>
-      <c r="F147" s="5" t="s">
-        <v>212</v>
-      </c>
+      <c r="A147" s="86"/>
+      <c r="B147" s="78"/>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A148" s="77"/>
-      <c r="B148" s="74"/>
-      <c r="C148" s="5" t="s">
-        <v>269</v>
-      </c>
-      <c r="D148" s="5" t="s">
-        <v>308</v>
-      </c>
-      <c r="F148" s="5" t="s">
-        <v>213</v>
+      <c r="A148" s="86"/>
+      <c r="B148" s="77" t="s">
+        <v>384</v>
+      </c>
+      <c r="C148" s="12" t="s">
+        <v>385</v>
+      </c>
+      <c r="D148" s="12" t="s">
+        <v>386</v>
+      </c>
+      <c r="E148" s="12"/>
+      <c r="F148" s="12" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A149" s="77"/>
-      <c r="B149" s="75"/>
-    </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A150" s="77"/>
-      <c r="B150" s="72" t="s">
+      <c r="A149" s="86"/>
+      <c r="B149" s="76"/>
+      <c r="C149" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="D149" s="5" t="s">
         <v>388</v>
       </c>
-      <c r="C150" s="12" t="s">
-        <v>389</v>
-      </c>
-      <c r="D150" s="12" t="s">
-        <v>390</v>
-      </c>
-      <c r="E150" s="12"/>
-      <c r="F150" s="12" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A151" s="77"/>
-      <c r="B151" s="73"/>
-      <c r="C151" s="5" t="s">
-        <v>391</v>
-      </c>
-      <c r="D151" s="5" t="s">
-        <v>392</v>
-      </c>
-      <c r="F151" s="5" t="s">
-        <v>273</v>
+      <c r="F149" s="5" t="s">
+        <v>271</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="B148:B149"/>
+    <mergeCell ref="B142:B147"/>
+    <mergeCell ref="A119:A149"/>
+    <mergeCell ref="B116:B118"/>
+    <mergeCell ref="B122:B128"/>
+    <mergeCell ref="B129:B141"/>
+    <mergeCell ref="B119:B121"/>
+    <mergeCell ref="A107:A118"/>
+    <mergeCell ref="B113:B115"/>
+    <mergeCell ref="B107:B109"/>
+    <mergeCell ref="B110:B112"/>
     <mergeCell ref="B84:B86"/>
     <mergeCell ref="A2:A45"/>
     <mergeCell ref="B2:B11"/>
@@ -5352,17 +5323,6 @@
     <mergeCell ref="B97:B106"/>
     <mergeCell ref="B78:B80"/>
     <mergeCell ref="B81:B83"/>
-    <mergeCell ref="B150:B151"/>
-    <mergeCell ref="B144:B149"/>
-    <mergeCell ref="A121:A151"/>
-    <mergeCell ref="B118:B120"/>
-    <mergeCell ref="B124:B130"/>
-    <mergeCell ref="B131:B143"/>
-    <mergeCell ref="B121:B123"/>
-    <mergeCell ref="A107:A120"/>
-    <mergeCell ref="B115:B117"/>
-    <mergeCell ref="B107:B110"/>
-    <mergeCell ref="B111:B114"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>